<commit_message>
feat: added URL parameter direct linking
</commit_message>
<xml_diff>
--- a/Pronoms_Relatifs.xlsx
+++ b/Pronoms_Relatifs.xlsx
@@ -428,17 +428,16 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -498,8 +497,14 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="1">
+  <tableStyles count="2">
     <tableStyle count="4" pivot="0" name="Pronoms Relatifs - Basique-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="Pronoms Relatifs - Avancé-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -528,6 +533,20 @@
     <tableColumn name="FeedbackIncorrect" id="6"/>
   </tableColumns>
   <tableStyleInfo name="Pronoms Relatifs - Basique-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F16" displayName="Table2" name="Table2" id="2">
+  <tableColumns count="6">
+    <tableColumn name="Type" id="1"/>
+    <tableColumn name="Question" id="2"/>
+    <tableColumn name="Options" id="3"/>
+    <tableColumn name="Answer" id="4"/>
+    <tableColumn name="FeedbackCorrect" id="5"/>
+    <tableColumn name="FeedbackIncorrect" id="6"/>
+  </tableColumns>
+  <tableStyleInfo name="Pronoms Relatifs - Avancé-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -787,6 +806,7 @@
       <c r="B3" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
@@ -804,6 +824,7 @@
       <c r="B4" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
         <v>19</v>
       </c>
@@ -821,6 +842,7 @@
       <c r="B5" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
         <v>23</v>
       </c>
@@ -878,6 +900,7 @@
       <c r="B8" s="2" t="s">
         <v>36</v>
       </c>
+      <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
         <v>9</v>
       </c>
@@ -895,6 +918,7 @@
       <c r="B9" s="2" t="s">
         <v>39</v>
       </c>
+      <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
         <v>19</v>
       </c>
@@ -932,6 +956,7 @@
       <c r="B11" s="2" t="s">
         <v>46</v>
       </c>
+      <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
         <v>23</v>
       </c>
@@ -969,6 +994,7 @@
       <c r="B13" s="2" t="s">
         <v>52</v>
       </c>
+      <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
         <v>14</v>
       </c>
@@ -986,6 +1012,7 @@
       <c r="B14" s="2" t="s">
         <v>55</v>
       </c>
+      <c r="C14" s="2"/>
       <c r="D14" s="2" t="s">
         <v>19</v>
       </c>
@@ -2034,302 +2061,315 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="26" width="8.71"/>
+    <col customWidth="1" min="1" max="1" width="16.43"/>
+    <col customWidth="1" min="2" max="2" width="43.0"/>
+    <col customWidth="1" min="3" max="3" width="37.14"/>
+    <col customWidth="1" min="4" max="4" width="23.29"/>
+    <col customWidth="1" min="5" max="6" width="43.0"/>
+    <col customWidth="1" min="7" max="26" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="22.5" customHeight="1">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="C3" s="2"/>
+      <c r="D3" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="C4" s="2"/>
+      <c r="D4" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="s">
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="C6" s="2"/>
+      <c r="D6" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="C7" s="2"/>
+      <c r="D7" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="s">
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="s">
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="C9" s="2"/>
+      <c r="D9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="s">
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="C10" s="2"/>
+      <c r="D10" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="s">
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="s">
+    <row r="12" ht="22.5" customHeight="1">
+      <c r="A12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="s">
+    <row r="13" ht="22.5" customHeight="1">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="C13" s="2"/>
+      <c r="D13" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="s">
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="s">
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="C15" s="2"/>
+      <c r="D15" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="s">
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="2" t="s">
         <v>125</v>
       </c>
     </row>
@@ -3318,5 +3358,8 @@
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: restore missing selectTopic and populateTopics logic
</commit_message>
<xml_diff>
--- a/Pronoms_Relatifs.xlsx
+++ b/Pronoms_Relatifs.xlsx
@@ -428,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -437,6 +437,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2070,306 +2076,306 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2" t="s">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="4" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="4" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="4" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="4" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="4" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="4" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="4" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="4" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2" t="s">
+      <c r="C13" s="4"/>
+      <c r="D13" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="4" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="4" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="4" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="4" t="s">
         <v>125</v>
       </c>
     </row>

</xml_diff>